<commit_message>
implementa feedback controlado e prepara deploy
</commit_message>
<xml_diff>
--- a/Plano de trabalho/acompanhamento-app-do-amor.xlsx
+++ b/Plano de trabalho/acompanhamento-app-do-amor.xlsx
@@ -109,7 +109,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>14/09/2026 18:36</t>
+          <t>16/09/2026 20:36</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -142,7 +142,7 @@
         </is>
       </c>
       <c r="B4" s="2">
-        <f>COUNTA('Plano Mestre'!A2:A138)</f>
+        <f>COUNTA('Plano Mestre'!A2:A140)</f>
         <v>0</v>
       </c>
       <c r="C4" s="0" t="inlineStr">
@@ -158,7 +158,7 @@
         </is>
       </c>
       <c r="B5" s="2">
-        <f>COUNTIF('Plano Mestre'!I2:I138,"Concluído")</f>
+        <f>COUNTIF('Plano Mestre'!I2:I140,"Concluído")</f>
         <v>0</v>
       </c>
       <c r="C5" s="0" t="inlineStr">
@@ -174,7 +174,7 @@
         </is>
       </c>
       <c r="B6" s="2">
-        <f>COUNTIF('Plano Mestre'!I2:I138,"Em andamento")</f>
+        <f>COUNTIF('Plano Mestre'!I2:I140,"Em andamento")</f>
         <v>0</v>
       </c>
       <c r="C6" s="0" t="inlineStr">
@@ -190,7 +190,7 @@
         </is>
       </c>
       <c r="B7" s="2">
-        <f>COUNTIF('Plano Mestre'!I2:I138,"Não iniciado")</f>
+        <f>COUNTIF('Plano Mestre'!I2:I140,"Não iniciado")</f>
         <v>0</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
@@ -206,7 +206,7 @@
         </is>
       </c>
       <c r="B8" s="3">
-        <f>AVERAGE('Plano Mestre'!M2:M138)</f>
+        <f>AVERAGE('Plano Mestre'!M2:M140)</f>
         <v>0</v>
       </c>
       <c r="C8" s="0" t="inlineStr">
@@ -222,7 +222,7 @@
         </is>
       </c>
       <c r="B9" s="2">
-        <f>SUM('Plano Mestre'!J2:J138)</f>
+        <f>SUM('Plano Mestre'!J2:J140)</f>
         <v>0</v>
       </c>
       <c r="C9" s="0" t="inlineStr">
@@ -272,11 +272,11 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B138,"Descoberta")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B140,"Descoberta")</f>
         <v>0</v>
       </c>
       <c r="C12" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B138,"Descoberta",'Plano Mestre'!I2:I138,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B140,"Descoberta",'Plano Mestre'!I2:I140,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -287,11 +287,11 @@
         </is>
       </c>
       <c r="B13" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B138,"Planejamento")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B140,"Planejamento")</f>
         <v>0</v>
       </c>
       <c r="C13" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B138,"Planejamento",'Plano Mestre'!I2:I138,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B140,"Planejamento",'Plano Mestre'!I2:I140,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -302,11 +302,11 @@
         </is>
       </c>
       <c r="B14" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B138,"Marca")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B140,"Marca")</f>
         <v>0</v>
       </c>
       <c r="C14" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B138,"Marca",'Plano Mestre'!I2:I138,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B140,"Marca",'Plano Mestre'!I2:I140,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -317,11 +317,11 @@
         </is>
       </c>
       <c r="B15" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B138,"UX/UI")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B140,"UX/UI")</f>
         <v>0</v>
       </c>
       <c r="C15" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B138,"UX/UI",'Plano Mestre'!I2:I138,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B140,"UX/UI",'Plano Mestre'!I2:I140,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -332,11 +332,11 @@
         </is>
       </c>
       <c r="B16" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B138,"Arquitetura")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B140,"Arquitetura")</f>
         <v>0</v>
       </c>
       <c r="C16" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B138,"Arquitetura",'Plano Mestre'!I2:I138,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B140,"Arquitetura",'Plano Mestre'!I2:I140,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -347,11 +347,11 @@
         </is>
       </c>
       <c r="B17" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B138,"Infraestrutura")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B140,"Infraestrutura")</f>
         <v>0</v>
       </c>
       <c r="C17" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B138,"Infraestrutura",'Plano Mestre'!I2:I138,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B140,"Infraestrutura",'Plano Mestre'!I2:I140,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -362,11 +362,11 @@
         </is>
       </c>
       <c r="B18" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B138,"Backend")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B140,"Backend")</f>
         <v>0</v>
       </c>
       <c r="C18" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B138,"Backend",'Plano Mestre'!I2:I138,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B140,"Backend",'Plano Mestre'!I2:I140,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -377,11 +377,11 @@
         </is>
       </c>
       <c r="B19" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B138,"Frontend")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B140,"Frontend")</f>
         <v>0</v>
       </c>
       <c r="C19" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B138,"Frontend",'Plano Mestre'!I2:I138,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B140,"Frontend",'Plano Mestre'!I2:I140,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -392,11 +392,11 @@
         </is>
       </c>
       <c r="B20" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B138,"Conteúdo")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B140,"Conteúdo")</f>
         <v>0</v>
       </c>
       <c r="C20" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B138,"Conteúdo",'Plano Mestre'!I2:I138,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B140,"Conteúdo",'Plano Mestre'!I2:I140,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -407,11 +407,11 @@
         </is>
       </c>
       <c r="B21" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B138,"Qualidade")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B140,"Qualidade")</f>
         <v>0</v>
       </c>
       <c r="C21" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B138,"Qualidade",'Plano Mestre'!I2:I138,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B140,"Qualidade",'Plano Mestre'!I2:I140,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -422,11 +422,11 @@
         </is>
       </c>
       <c r="B22" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B138,"Jurídico")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B140,"Jurídico")</f>
         <v>0</v>
       </c>
       <c r="C22" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B138,"Jurídico",'Plano Mestre'!I2:I138,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B140,"Jurídico",'Plano Mestre'!I2:I140,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -437,11 +437,11 @@
         </is>
       </c>
       <c r="B23" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B138,"Lançamento")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B140,"Lançamento")</f>
         <v>0</v>
       </c>
       <c r="C23" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B138,"Lançamento",'Plano Mestre'!I2:I138,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B140,"Lançamento",'Plano Mestre'!I2:I140,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -452,11 +452,11 @@
         </is>
       </c>
       <c r="B24" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B138,"Pós-lançamento")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B140,"Pós-lançamento")</f>
         <v>0</v>
       </c>
       <c r="C24" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B138,"Pós-lançamento",'Plano Mestre'!I2:I138,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B140,"Pós-lançamento",'Plano Mestre'!I2:I140,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -467,11 +467,11 @@
         </is>
       </c>
       <c r="B25" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B138,"MPV de teste")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B140,"MPV de teste")</f>
         <v>0</v>
       </c>
       <c r="C25" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B138,"MPV de teste",'Plano Mestre'!I2:I138,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B140,"MPV de teste",'Plano Mestre'!I2:I140,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -3384,7 +3384,7 @@
       </c>
       <c r="I44" s="0" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="J44" s="0">
@@ -3401,11 +3401,11 @@
         </is>
       </c>
       <c r="M44" s="3">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="N44" s="0" t="inlineStr">
         <is>
-          <t>Separar logs métricas e alertas por ambiente e versão conforme docs/AMBIENTES.md - implementar sondas de saúde e prontidão sem dados privados - testar alertas de indisponibilidade erros banco backup e capacidade sem conteúdo íntimo ou segredos</t>
+          <t>Sonda mínima GET /api/health implementada sem dados privados em 16/09/2026 - ainda separar logs métricas e alertas por ambiente e versão implementar prontidão do armazenamento e testar alertas de indisponibilidade erros banco backup e capacidade sem conteúdo íntimo ou segredos</t>
         </is>
       </c>
     </row>
@@ -8883,7 +8883,7 @@
       </c>
       <c r="N127" s="0" t="inlineStr">
         <is>
-          <t>Fluxo aprovado em docs/FLUXO-MPV.md com seis estados entrada direta dois jogos de três rodadas feedback de três sinais exceções e critérios de aceite — concluído antecipadamente em 12/09/2026</t>
+          <t>Fluxo aprovado em docs/FLUXO-MPV.md com seis estados entrada direta dois jogos de três rodadas três sinais e sugestão opcional exceções e critérios de aceite — atualizado em 16/09/2026</t>
         </is>
       </c>
     </row>
@@ -9213,7 +9213,7 @@
       </c>
       <c r="N132" s="0" t="inlineStr">
         <is>
-          <t>Feedback binário compartilhado implementado nos dois jogos com registro local somente do jogo concluído, clareza, descoberta ou conexão e intenção de jogar novamente, sem conteúdo das rodadas — concluído antecipadamente em 12/09/2026</t>
+          <t>Feedback binário compartilhado implementado nos dois jogos e integrado ao registro central do jogo concluído clareza descoberta ou conexão e intenção de jogar novamente sem conteúdo das rodadas — concluído antecipadamente em 12/09/2026 e integrado em 16/09/2026</t>
         </is>
       </c>
     </row>
@@ -9380,7 +9380,7 @@
       </c>
       <c r="G135" s="0" t="inlineStr">
         <is>
-          <t>132,133</t>
+          <t>132,133,138,139</t>
         </is>
       </c>
       <c r="H135" s="0" t="inlineStr">
@@ -9411,7 +9411,7 @@
       </c>
       <c r="N135" s="0" t="inlineStr">
         <is>
-          <t>Validador móvel já cobre caminhos felizes pulo limpeza de escolha reinício e cancelamento de saída — iniciar aceite formal após concluir 132 e 133 e confirmar troca entre jogos sem estado residual</t>
+          <t>Validadores cobrem caminhos felizes pulo limpeza de escolha reinício cancelamento de saída sugestão opcional persistência exportação e serviço integrado de produção — iniciar aceite formal após concluir 132 e 133 e confirmar troca entre jogos sem estado residual</t>
         </is>
       </c>
     </row>
@@ -9456,7 +9456,7 @@
       </c>
       <c r="I136" s="0" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="J136" s="0">
@@ -9464,20 +9464,20 @@
       </c>
       <c r="K136" s="0" t="inlineStr">
         <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="L136" s="0" t="inlineStr">
+        <is>
           <t>22/09/2026</t>
         </is>
       </c>
-      <c r="L136" s="0" t="inlineStr">
-        <is>
-          <t>22/09/2026</t>
-        </is>
-      </c>
       <c r="M136" s="3">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="N136" s="0" t="inlineStr">
         <is>
-          <t>Publicação temporária sem cadastro dados pessoais analytics de terceiros ou indexação pública</t>
+          <t>Serviço único preparado e Blueprint do Render definido na região Virginia com plano pago disco persistente de 1 GB sonda de saúde CORS restrito bloqueio de indexação e segredo gerado — aguardando autenticação do workspace deploy HTTPS e validação do endereço final</t>
         </is>
       </c>
     </row>
@@ -9543,7 +9543,7 @@
       </c>
       <c r="N137" s="0" t="inlineStr">
         <is>
-          <t>Cada casal joga sem mediação e envia apenas os três sinais do produto — não há entrevistas nem etapa de pesquisa dentro do MPV</t>
+          <t>Cada casal joga sem mediação e envia os três sinais do produto com sugestão de melhoria opcional — não há entrevistas nem etapa de pesquisa dentro do MPV</t>
         </is>
       </c>
     </row>
@@ -9613,8 +9613,140 @@
         </is>
       </c>
     </row>
+    <row r="139">
+      <c r="A139" s="0">
+        <v>138</v>
+      </c>
+      <c r="B139" s="0" t="inlineStr">
+        <is>
+          <t>MPV de teste</t>
+        </is>
+      </c>
+      <c r="C139" s="0" t="inlineStr">
+        <is>
+          <t>Feedback</t>
+        </is>
+      </c>
+      <c r="D139" s="0" t="inlineStr">
+        <is>
+          <t>Adicionar sugestões abertas opcionais ao feedback</t>
+        </is>
+      </c>
+      <c r="E139" s="0" t="inlineStr">
+        <is>
+          <t>Campo de sugestões funcional</t>
+        </is>
+      </c>
+      <c r="F139" s="0" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G139" s="0" t="inlineStr">
+        <is>
+          <t>131</t>
+        </is>
+      </c>
+      <c r="H139" s="0" t="inlineStr">
+        <is>
+          <t>Engenharia Frontend</t>
+        </is>
+      </c>
+      <c r="I139" s="0" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="J139" s="0">
+        <v>3</v>
+      </c>
+      <c r="K139" s="0" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="L139" s="0" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="M139" s="3">
+        <v>1</v>
+      </c>
+      <c r="N139" s="0" t="inlineStr">
+        <is>
+          <t>Campo opcional de até 500 caracteres implementado com orientação para não inserir dados pessoais e cobertura na matriz móvel — concluído em 16/09/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="0">
+        <v>139</v>
+      </c>
+      <c r="B140" s="0" t="inlineStr">
+        <is>
+          <t>MPV de teste</t>
+        </is>
+      </c>
+      <c r="C140" s="0" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="D140" s="0" t="inlineStr">
+        <is>
+          <t>Centralizar feedback e disponibilizar exportação controlada</t>
+        </is>
+      </c>
+      <c r="E140" s="0" t="inlineStr">
+        <is>
+          <t>API e CSV protegidos</t>
+        </is>
+      </c>
+      <c r="F140" s="0" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+      <c r="G140" s="0" t="inlineStr">
+        <is>
+          <t>138</t>
+        </is>
+      </c>
+      <c r="H140" s="0" t="inlineStr">
+        <is>
+          <t>Engenharia Backend</t>
+        </is>
+      </c>
+      <c r="I140" s="0" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="J140" s="0">
+        <v>6</v>
+      </c>
+      <c r="K140" s="0" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="L140" s="0" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="M140" s="3">
+        <v>1</v>
+      </c>
+      <c r="N140" s="0" t="inlineStr">
+        <is>
+          <t>POST anônimo com validação idempotência controle de origem rate limit e retenção no JSON além de exportação CSV protegida por token e testes automatizados — concluído em 16/09/2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N138"/>
+  <autoFilter ref="A1:N140"/>
   <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>
@@ -11017,8 +11149,50 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>MR06</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>Sugestão aberta conter nomes contatos ou detalhes pessoais</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>Privacidade</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>Média</t>
+        </is>
+      </c>
+      <c r="E21" s="0" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="F21" s="0" t="inlineStr">
+        <is>
+          <t>Limitar a 500 caracteres orientar a não inserir dados pessoais restringir a exportação e aplicar retenção de 90 dias</t>
+        </is>
+      </c>
+      <c r="G21" s="0" t="inlineStr">
+        <is>
+          <t>Privacidade/Jurídico</t>
+        </is>
+      </c>
+      <c r="H21" s="0" t="inlineStr">
+        <is>
+          <t>Aberto</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H20"/>
+  <autoFilter ref="A1:H21"/>
   <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
configura origem do deploy no Render
</commit_message>
<xml_diff>
--- a/Plano de trabalho/acompanhamento-app-do-amor.xlsx
+++ b/Plano de trabalho/acompanhamento-app-do-amor.xlsx
@@ -109,7 +109,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>16/09/2026 20:36</t>
+          <t>16/09/2026 20:39</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -9477,7 +9477,7 @@
       </c>
       <c r="N136" s="0" t="inlineStr">
         <is>
-          <t>Serviço único preparado e Blueprint do Render definido na região Virginia com plano pago disco persistente de 1 GB sonda de saúde CORS restrito bloqueio de indexação e segredo gerado — aguardando autenticação do workspace deploy HTTPS e validação do endereço final</t>
+          <t>Serviço único preparado e Blueprint do Render definido na região Virginia com plano pago disco persistente de 1 GB sonda de saúde CORS restrito bloqueio de indexação e segredo gerado — workspace autenticado e aguardando cadastro de pagamento deploy HTTPS e validação do endereço final</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
usa PostgreSQL gratuito para feedback do MPV
</commit_message>
<xml_diff>
--- a/Plano de trabalho/acompanhamento-app-do-amor.xlsx
+++ b/Plano de trabalho/acompanhamento-app-do-amor.xlsx
@@ -109,7 +109,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>16/09/2026 20:39</t>
+          <t>16/09/2026 20:47</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -2943,7 +2943,7 @@
       </c>
       <c r="N37" s="0" t="inlineStr">
         <is>
-          <t>Baseline STRIDE e OWASP em docs/MODELAGEM-DE-AMEACAS.md com diagrama ativos fronteiras 22 ameaças 29 controles 20 testes gates de piloto e riscos residuais - 13 ameaças críticas 8 altas e 1 média - estado atual não apto para piloto externo - revalidar após tarefas 112-114 PostgreSQL provedores e antes da release candidate</t>
+          <t>Baseline STRIDE e OWASP em docs/MODELAGEM-DE-AMEACAS.md com diagrama ativos fronteiras 23 ameaças 30 controles 21 testes gates de piloto e riscos residuais - 13 ameaças críticas 9 altas e 1 média - estado atual não apto para piloto externo - revalidar após tarefas 112-114 PostgreSQL provedores e antes da release candidate</t>
         </is>
       </c>
     </row>
@@ -3252,7 +3252,7 @@
       </c>
       <c r="I42" s="0" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="J42" s="0">
@@ -3269,11 +3269,11 @@
         </is>
       </c>
       <c r="M42" s="3">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="N42" s="0" t="inlineStr">
         <is>
-          <t>Provisionar PostgreSQL local staging e production com identidades distintas mesma versão principal e migrações conforme docs/AMBIENTES.md - implementar DATABASE_URL validar conexão integridade e concorrência - JSON atual sem transações fica restrito ao protótipo local</t>
+          <t>Adaptador DATABASE_URL e schema idempotente implementados para o feedback do MPV em 16/09/2026 com PostgreSQL gratuito temporário no Render - ainda provisionar local staging e production definitivos com identidades distintas migrações integridade concorrência e migração dos demais dados</t>
         </is>
       </c>
     </row>
@@ -9477,7 +9477,7 @@
       </c>
       <c r="N136" s="0" t="inlineStr">
         <is>
-          <t>Serviço único preparado e Blueprint do Render definido na região Virginia com plano pago disco persistente de 1 GB sonda de saúde CORS restrito bloqueio de indexação e segredo gerado — workspace autenticado e aguardando cadastro de pagamento deploy HTTPS e validação do endereço final</t>
+          <t>Blueprint gratuito do Render definido na região Virginia com Web Service PostgreSQL de 1 GB sonda de saúde CORS restrito bloqueio de indexação e segredo gerado — banco expira em 30 dias sem backup e aguardam deploy HTTPS exportação de teste e validação do endereço final</t>
         </is>
       </c>
     </row>
@@ -9741,7 +9741,7 @@
       </c>
       <c r="N140" s="0" t="inlineStr">
         <is>
-          <t>POST anônimo com validação idempotência controle de origem rate limit e retenção no JSON além de exportação CSV protegida por token e testes automatizados — concluído em 16/09/2026</t>
+          <t>POST anônimo com validação idempotência controle de origem rate limit armazenamento PostgreSQL remoto com fallback JSON local e exportação CSV protegida por token — concluído em 16/09/2026</t>
         </is>
       </c>
     </row>
@@ -10589,7 +10589,7 @@
       </c>
       <c r="F7" s="0" t="inlineStr">
         <is>
-          <t>Migrar para PostgreSQL antes da publicação</t>
+          <t>Feedback remoto já usa PostgreSQL temporário - migrar os demais dados e provisionar banco definitivo antes da publicação ampla</t>
         </is>
       </c>
       <c r="G7" s="0" t="inlineStr">
@@ -11177,7 +11177,7 @@
       </c>
       <c r="F21" s="0" t="inlineStr">
         <is>
-          <t>Limitar a 500 caracteres orientar a não inserir dados pessoais restringir a exportação e aplicar retenção de 90 dias</t>
+          <t>Limitar a 500 caracteres orientar a não inserir dados pessoais restringir a exportação e excluir a base gratuita em até 30 dias</t>
         </is>
       </c>
       <c r="G21" s="0" t="inlineStr">

</xml_diff>

<commit_message>
registra publicacao gratuita do teste
</commit_message>
<xml_diff>
--- a/Plano de trabalho/acompanhamento-app-do-amor.xlsx
+++ b/Plano de trabalho/acompanhamento-app-do-amor.xlsx
@@ -109,7 +109,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>16/09/2026 20:47</t>
+          <t>16/09/2026 20:55</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -9456,7 +9456,7 @@
       </c>
       <c r="I136" s="0" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="J136" s="0">
@@ -9469,15 +9469,15 @@
       </c>
       <c r="L136" s="0" t="inlineStr">
         <is>
-          <t>22/09/2026</t>
+          <t>16/09/2026</t>
         </is>
       </c>
       <c r="M136" s="3">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="N136" s="0" t="inlineStr">
         <is>
-          <t>Blueprint gratuito do Render definido na região Virginia com Web Service PostgreSQL de 1 GB sonda de saúde CORS restrito bloqueio de indexação e segredo gerado — banco expira em 30 dias sem backup e aguardam deploy HTTPS exportação de teste e validação do endereço final</t>
+          <t>Demonstração HTTPS publicada no Render gratuito com Web Service PostgreSQL de 1 GB sonda de saúde CORS restrito bloqueio de indexação e segredo operacional — envio persistência e exportação validados base sintética removida e banco expira em 16/10/2026 sem backup — passagem física Android e iPhone continua na tarefa 132 antes de ampliar o teste</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
inclui passagem fisica da tarefa 132
</commit_message>
<xml_diff>
--- a/Plano de trabalho/acompanhamento-app-do-amor.xlsx
+++ b/Plano de trabalho/acompanhamento-app-do-amor.xlsx
@@ -109,7 +109,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>16/09/2026 20:55</t>
+          <t>16/09/2026 21:01</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -9279,7 +9279,7 @@
       </c>
       <c r="N133" s="0" t="inlineStr">
         <is>
-          <t>Matriz Chromium revalidada em 14/09/2026 com cinco viewports e 95 estados em docs/VALIDACAO-MOBILE-MPV-2026-09-14.md — MOB-01 a MOB-03 resolvidos, sem overflow ou exposição do nome do aplicativo e com toque pulo confirmação rotação fluxos completos e reinício aprovados — pendente somente passagem física em Chrome Android e Safari iOS</t>
+          <t>Matriz Chromium revalidada em 14/09/2026 com cinco viewports e 95 estados — roteiro físico incorporado em docs/VALIDACAO-MOBILE-MPV-2026-09-14.md com 12 verificações por plataforma identificação dos aparelhos evidências feedbacks técnicos e critério de aceite — pendente executar e registrar aprovação em Chrome Android e Safari iOS físicos e remover os dois feedbacks técnicos</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
registra aceite fisico no Chrome
</commit_message>
<xml_diff>
--- a/Plano de trabalho/acompanhamento-app-do-amor.xlsx
+++ b/Plano de trabalho/acompanhamento-app-do-amor.xlsx
@@ -109,7 +109,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>16/09/2026 21:01</t>
+          <t>16/09/2026 21:11</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -9258,7 +9258,7 @@
       </c>
       <c r="I133" s="0" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="J133" s="0">
@@ -9266,20 +9266,20 @@
       </c>
       <c r="K133" s="0" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>16/09/2026</t>
         </is>
       </c>
       <c r="L133" s="0" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>16/09/2026</t>
         </is>
       </c>
       <c r="M133" s="3">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="N133" s="0" t="inlineStr">
         <is>
-          <t>Matriz Chromium revalidada em 14/09/2026 com cinco viewports e 95 estados — roteiro físico incorporado em docs/VALIDACAO-MOBILE-MPV-2026-09-14.md com 12 verificações por plataforma identificação dos aparelhos evidências feedbacks técnicos e critério de aceite — pendente executar e registrar aprovação em Chrome Android e Safari iOS físicos e remover os dois feedbacks técnicos</t>
+          <t>Aprovado com ressalva para o escopo controlado no Chrome após passagem física confirmada pela Product Owner feedback real com três sinais positivos saúde exportação persistência dois jogos e 95 estados móveis revalidados — registro técnico removido e base vazia — modelo sistema e versão não informados — Safari adiado por decisão da Product Owner e explicitamente não validado</t>
         </is>
       </c>
     </row>
@@ -9390,7 +9390,7 @@
       </c>
       <c r="I135" s="0" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="J135" s="0">
@@ -9398,20 +9398,20 @@
       </c>
       <c r="K135" s="0" t="inlineStr">
         <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="L135" s="0" t="inlineStr">
+        <is>
           <t>21/09/2026</t>
         </is>
       </c>
-      <c r="L135" s="0" t="inlineStr">
-        <is>
-          <t>21/09/2026</t>
-        </is>
-      </c>
       <c r="M135" s="3">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="N135" s="0" t="inlineStr">
         <is>
-          <t>Validadores cobrem caminhos felizes pulo limpeza de escolha reinício cancelamento de saída sugestão opcional persistência exportação e serviço integrado de produção — iniciar aceite formal após concluir 132 e 133 e confirmar troca entre jogos sem estado residual</t>
+          <t>API serviço integrado e matriz móvel revalidados com sucesso em 16/09/2026 após a passagem física no Chrome — pendem concluir as verificações formais de acessibilidade da tarefa 133 e registrar o aceite final — Safari permanece fora da cobertura atual</t>
         </is>
       </c>
     </row>
@@ -9477,7 +9477,7 @@
       </c>
       <c r="N136" s="0" t="inlineStr">
         <is>
-          <t>Demonstração HTTPS publicada no Render gratuito com Web Service PostgreSQL de 1 GB sonda de saúde CORS restrito bloqueio de indexação e segredo operacional — envio persistência e exportação validados base sintética removida e banco expira em 16/10/2026 sem backup — passagem física Android e iPhone continua na tarefa 132 antes de ampliar o teste</t>
+          <t>Demonstração HTTPS publicada no Render gratuito com Web Service PostgreSQL de 1 GB sonda de saúde CORS restrito bloqueio de indexação e segredo operacional — envio persistência exportação e passagem física no Chrome validados base técnica limpa e banco expira em 16/10/2026 sem backup — Safari permanece fora da cobertura atual</t>
         </is>
       </c>
     </row>
@@ -9851,7 +9851,7 @@
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="E3" s="0" t="inlineStr">
@@ -9886,12 +9886,12 @@
       </c>
       <c r="D4" s="0" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="E4" s="0" t="inlineStr">
         <is>
-          <t>QA crítico aprovado e link controlado disponível</t>
+          <t>Link controlado disponível e QA em curso com aceite físico restrito ao Chrome</t>
         </is>
       </c>
       <c r="F4" s="0" t="inlineStr">

</xml_diff>

<commit_message>
adiciona amostra afetiva e baralho visual
</commit_message>
<xml_diff>
--- a/Plano de trabalho/acompanhamento-app-do-amor.xlsx
+++ b/Plano de trabalho/acompanhamento-app-do-amor.xlsx
@@ -109,7 +109,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>16/09/2026 21:11</t>
+          <t>17/09/2026 12:29</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -142,7 +142,7 @@
         </is>
       </c>
       <c r="B4" s="2">
-        <f>COUNTA('Plano Mestre'!A2:A140)</f>
+        <f>COUNTA('Plano Mestre'!A2:A143)</f>
         <v>0</v>
       </c>
       <c r="C4" s="0" t="inlineStr">
@@ -158,7 +158,7 @@
         </is>
       </c>
       <c r="B5" s="2">
-        <f>COUNTIF('Plano Mestre'!I2:I140,"Concluído")</f>
+        <f>COUNTIF('Plano Mestre'!I2:I143,"Concluído")</f>
         <v>0</v>
       </c>
       <c r="C5" s="0" t="inlineStr">
@@ -174,7 +174,7 @@
         </is>
       </c>
       <c r="B6" s="2">
-        <f>COUNTIF('Plano Mestre'!I2:I140,"Em andamento")</f>
+        <f>COUNTIF('Plano Mestre'!I2:I143,"Em andamento")</f>
         <v>0</v>
       </c>
       <c r="C6" s="0" t="inlineStr">
@@ -190,7 +190,7 @@
         </is>
       </c>
       <c r="B7" s="2">
-        <f>COUNTIF('Plano Mestre'!I2:I140,"Não iniciado")</f>
+        <f>COUNTIF('Plano Mestre'!I2:I143,"Não iniciado")</f>
         <v>0</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
@@ -206,7 +206,7 @@
         </is>
       </c>
       <c r="B8" s="3">
-        <f>AVERAGE('Plano Mestre'!M2:M140)</f>
+        <f>AVERAGE('Plano Mestre'!M2:M143)</f>
         <v>0</v>
       </c>
       <c r="C8" s="0" t="inlineStr">
@@ -222,7 +222,7 @@
         </is>
       </c>
       <c r="B9" s="2">
-        <f>SUM('Plano Mestre'!J2:J140)</f>
+        <f>SUM('Plano Mestre'!J2:J143)</f>
         <v>0</v>
       </c>
       <c r="C9" s="0" t="inlineStr">
@@ -272,11 +272,11 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B140,"Descoberta")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B143,"Descoberta")</f>
         <v>0</v>
       </c>
       <c r="C12" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B140,"Descoberta",'Plano Mestre'!I2:I140,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B143,"Descoberta",'Plano Mestre'!I2:I143,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -287,11 +287,11 @@
         </is>
       </c>
       <c r="B13" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B140,"Planejamento")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B143,"Planejamento")</f>
         <v>0</v>
       </c>
       <c r="C13" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B140,"Planejamento",'Plano Mestre'!I2:I140,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B143,"Planejamento",'Plano Mestre'!I2:I143,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -302,11 +302,11 @@
         </is>
       </c>
       <c r="B14" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B140,"Marca")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B143,"Marca")</f>
         <v>0</v>
       </c>
       <c r="C14" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B140,"Marca",'Plano Mestre'!I2:I140,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B143,"Marca",'Plano Mestre'!I2:I143,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -317,11 +317,11 @@
         </is>
       </c>
       <c r="B15" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B140,"UX/UI")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B143,"UX/UI")</f>
         <v>0</v>
       </c>
       <c r="C15" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B140,"UX/UI",'Plano Mestre'!I2:I140,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B143,"UX/UI",'Plano Mestre'!I2:I143,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -332,11 +332,11 @@
         </is>
       </c>
       <c r="B16" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B140,"Arquitetura")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B143,"Arquitetura")</f>
         <v>0</v>
       </c>
       <c r="C16" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B140,"Arquitetura",'Plano Mestre'!I2:I140,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B143,"Arquitetura",'Plano Mestre'!I2:I143,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -347,11 +347,11 @@
         </is>
       </c>
       <c r="B17" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B140,"Infraestrutura")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B143,"Infraestrutura")</f>
         <v>0</v>
       </c>
       <c r="C17" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B140,"Infraestrutura",'Plano Mestre'!I2:I140,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B143,"Infraestrutura",'Plano Mestre'!I2:I143,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -362,11 +362,11 @@
         </is>
       </c>
       <c r="B18" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B140,"Backend")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B143,"Backend")</f>
         <v>0</v>
       </c>
       <c r="C18" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B140,"Backend",'Plano Mestre'!I2:I140,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B143,"Backend",'Plano Mestre'!I2:I143,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -377,11 +377,11 @@
         </is>
       </c>
       <c r="B19" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B140,"Frontend")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B143,"Frontend")</f>
         <v>0</v>
       </c>
       <c r="C19" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B140,"Frontend",'Plano Mestre'!I2:I140,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B143,"Frontend",'Plano Mestre'!I2:I143,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -392,11 +392,11 @@
         </is>
       </c>
       <c r="B20" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B140,"Conteúdo")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B143,"Conteúdo")</f>
         <v>0</v>
       </c>
       <c r="C20" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B140,"Conteúdo",'Plano Mestre'!I2:I140,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B143,"Conteúdo",'Plano Mestre'!I2:I143,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -407,11 +407,11 @@
         </is>
       </c>
       <c r="B21" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B140,"Qualidade")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B143,"Qualidade")</f>
         <v>0</v>
       </c>
       <c r="C21" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B140,"Qualidade",'Plano Mestre'!I2:I140,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B143,"Qualidade",'Plano Mestre'!I2:I143,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -422,11 +422,11 @@
         </is>
       </c>
       <c r="B22" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B140,"Jurídico")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B143,"Jurídico")</f>
         <v>0</v>
       </c>
       <c r="C22" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B140,"Jurídico",'Plano Mestre'!I2:I140,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B143,"Jurídico",'Plano Mestre'!I2:I143,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -437,11 +437,11 @@
         </is>
       </c>
       <c r="B23" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B140,"Lançamento")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B143,"Lançamento")</f>
         <v>0</v>
       </c>
       <c r="C23" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B140,"Lançamento",'Plano Mestre'!I2:I140,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B143,"Lançamento",'Plano Mestre'!I2:I143,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -452,11 +452,11 @@
         </is>
       </c>
       <c r="B24" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B140,"Pós-lançamento")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B143,"Pós-lançamento")</f>
         <v>0</v>
       </c>
       <c r="C24" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B140,"Pós-lançamento",'Plano Mestre'!I2:I140,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B143,"Pós-lançamento",'Plano Mestre'!I2:I143,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -467,11 +467,11 @@
         </is>
       </c>
       <c r="B25" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B140,"MPV de teste")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B143,"MPV de teste")</f>
         <v>0</v>
       </c>
       <c r="C25" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B140,"MPV de teste",'Plano Mestre'!I2:I140,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B143,"MPV de teste",'Plano Mestre'!I2:I143,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -8817,7 +8817,7 @@
       </c>
       <c r="N126" s="0" t="inlineStr">
         <is>
-          <t>Somente Descoberta a Dois e Adivinhe de Mim — sem pesquisa prévia cadastro pareamento remoto backend ou testes de personalidade neste teste</t>
+          <t>Escopo inicial de Descoberta a Dois e Adivinhe de Mim concluído — exceção posterior autorizada pela Product Owner em 17/09/2026 adiciona amostra autoral e baralho visual nas tarefas 140 e 141</t>
         </is>
       </c>
     </row>
@@ -8875,7 +8875,7 @@
       </c>
       <c r="L127" s="0" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="M127" s="3">
@@ -8883,7 +8883,7 @@
       </c>
       <c r="N127" s="0" t="inlineStr">
         <is>
-          <t>Fluxo aprovado em docs/FLUXO-MPV.md com seis estados entrada direta dois jogos de três rodadas três sinais e sugestão opcional exceções e critérios de aceite — atualizado em 16/09/2026</t>
+          <t>Fluxo ampliado em docs/FLUXO-MPV.md com entrada direta três experiências cartas fechadas dois jogos amostra individual três sinais sugestão opcional exceções e critérios de aceite</t>
         </is>
       </c>
     </row>
@@ -9007,7 +9007,7 @@
       </c>
       <c r="L129" s="0" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="M129" s="3">
@@ -9015,7 +9015,7 @@
       </c>
       <c r="N129" s="0" t="inlineStr">
         <is>
-          <t>Entrada direta responsiva com seleção e instruções dos dois jogos implementada sem cadastro ou pareamento, com apresentação neutra sem o nome do aplicativo em título metadados cabeçalho ou rodapé e com o aplicativo completo preservado em src/App.tsx — atualizado em 14/09/2026</t>
+          <t>Entrada direta responsiva ampliada para três experiências sem cadastro ou pareamento com apresentação neutra sem o nome do aplicativo em título metadados cabeçalho ou rodapé e aplicativo completo preservado — atualizada em 17/09/2026</t>
         </is>
       </c>
     </row>
@@ -9205,7 +9205,7 @@
       </c>
       <c r="L132" s="0" t="inlineStr">
         <is>
-          <t>19/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="M132" s="3">
@@ -9213,7 +9213,7 @@
       </c>
       <c r="N132" s="0" t="inlineStr">
         <is>
-          <t>Feedback binário compartilhado implementado nos dois jogos e integrado ao registro central do jogo concluído clareza descoberta ou conexão e intenção de jogar novamente sem conteúdo das rodadas — concluído antecipadamente em 12/09/2026 e integrado em 16/09/2026</t>
+          <t>Feedback binário integrado aos dois jogos e à amostra individual com textos adaptados e registro central de clareza reflexão ou conexão e intenção de repetir sem respostas das rodadas — ampliado em 17/09/2026</t>
         </is>
       </c>
     </row>
@@ -9345,7 +9345,7 @@
       </c>
       <c r="N134" s="0" t="inlineStr">
         <is>
-          <t>MOB-03 resolvido em 14/09/2026 com todos os alvos visíveis em pelo menos 44 px e nomes acessíveis aprovados na matriz móvel — pendentes validações formais de foco contraste e redução de movimento</t>
+          <t>Todos os alvos incluindo cartas fechadas permanecem com pelo menos 44 px e nomes acessíveis aprovados em 185 estados móveis — pendentes validações formais de foco contraste e redução de movimento</t>
         </is>
       </c>
     </row>
@@ -9411,7 +9411,7 @@
       </c>
       <c r="N135" s="0" t="inlineStr">
         <is>
-          <t>API serviço integrado e matriz móvel revalidados com sucesso em 16/09/2026 após a passagem física no Chrome — pendem concluir as verificações formais de acessibilidade da tarefa 133 e registrar o aceite final — Safari permanece fora da cobertura atual</t>
+          <t>API serviço integrado três experiências baralho visual e matriz de 185 estados revalidados automaticamente em 17/09/2026 — pendem verificações formais da tarefa 133 e nova passagem física da tarefa 142 — Safari fora da cobertura atual</t>
         </is>
       </c>
     </row>
@@ -9512,7 +9512,7 @@
       </c>
       <c r="G137" s="0" t="inlineStr">
         <is>
-          <t>135</t>
+          <t>135,142</t>
         </is>
       </c>
       <c r="H137" s="0" t="inlineStr">
@@ -9543,7 +9543,7 @@
       </c>
       <c r="N137" s="0" t="inlineStr">
         <is>
-          <t>Cada casal joga sem mediação e envia os três sinais do produto com sugestão de melhoria opcional — não há entrevistas nem etapa de pesquisa dentro do MPV</t>
+          <t>Cada casal usa as experiências sem mediação e envia os três sinais do produto com sugestão de melhoria opcional — não há entrevistas nem etapa de pesquisa dentro do MPV — iniciar após a nova passagem física da versão ampliada</t>
         </is>
       </c>
     </row>
@@ -9745,8 +9745,206 @@
         </is>
       </c>
     </row>
+    <row r="141">
+      <c r="A141" s="0">
+        <v>140</v>
+      </c>
+      <c r="B141" s="0" t="inlineStr">
+        <is>
+          <t>MPV de teste</t>
+        </is>
+      </c>
+      <c r="C141" s="0" t="inlineStr">
+        <is>
+          <t>Experimento</t>
+        </is>
+      </c>
+      <c r="D141" s="0" t="inlineStr">
+        <is>
+          <t>Adicionar amostra autoral de preferências afetivas</t>
+        </is>
+      </c>
+      <c r="E141" s="0" t="inlineStr">
+        <is>
+          <t>Amostra individual funcional</t>
+        </is>
+      </c>
+      <c r="F141" s="0" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G141" s="0" t="inlineStr">
+        <is>
+          <t>126,128,139</t>
+        </is>
+      </c>
+      <c r="H141" s="0" t="inlineStr">
+        <is>
+          <t>Engenharia Frontend</t>
+        </is>
+      </c>
+      <c r="I141" s="0" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="J141" s="0">
+        <v>10</v>
+      </c>
+      <c r="K141" s="0" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="L141" s="0" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="M141" s="3">
+        <v>1</v>
+      </c>
+      <c r="N141" s="0" t="inlineStr">
+        <is>
+          <t>Cinco perguntas sorteadas entre seis situações autorais com cinco famílias de preferência pontuação somente em memória resultado com duas preferências fortes distribuição completa aviso não oficial e feedback adaptado — conteúdo não replica questionários comerciais</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="0">
+        <v>141</v>
+      </c>
+      <c r="B142" s="0" t="inlineStr">
+        <is>
+          <t>MPV de teste</t>
+        </is>
+      </c>
+      <c r="C142" s="0" t="inlineStr">
+        <is>
+          <t>UX</t>
+        </is>
+      </c>
+      <c r="D142" s="0" t="inlineStr">
+        <is>
+          <t>Apresentar perguntas como cartas fechadas escolhidas pela pessoa</t>
+        </is>
+      </c>
+      <c r="E142" s="0" t="inlineStr">
+        <is>
+          <t>Baralho visual acessível</t>
+        </is>
+      </c>
+      <c r="F142" s="0" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G142" s="0" t="inlineStr">
+        <is>
+          <t>129,130,140</t>
+        </is>
+      </c>
+      <c r="H142" s="0" t="inlineStr">
+        <is>
+          <t>Engenharia Frontend</t>
+        </is>
+      </c>
+      <c r="I142" s="0" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="J142" s="0">
+        <v>8</v>
+      </c>
+      <c r="K142" s="0" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="L142" s="0" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="M142" s="3">
+        <v>1</v>
+      </c>
+      <c r="N142" s="0" t="inlineStr">
+        <is>
+          <t>Componente visual em HTML e CSS aplicado às três experiências com escolha real entre cartas restantes animação rótulos acessíveis alvos mínimos de 44 px redução de movimento e reinício validado</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="0">
+        <v>142</v>
+      </c>
+      <c r="B143" s="0" t="inlineStr">
+        <is>
+          <t>MPV de teste</t>
+        </is>
+      </c>
+      <c r="C143" s="0" t="inlineStr">
+        <is>
+          <t>Qualidade</t>
+        </is>
+      </c>
+      <c r="D143" s="0" t="inlineStr">
+        <is>
+          <t>Revalidar versão ampliada e repetir passagem física no Chrome</t>
+        </is>
+      </c>
+      <c r="E143" s="0" t="inlineStr">
+        <is>
+          <t>Aceite da iteração ampliada</t>
+        </is>
+      </c>
+      <c r="F143" s="0" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+      <c r="G143" s="0" t="inlineStr">
+        <is>
+          <t>133,134,140,141</t>
+        </is>
+      </c>
+      <c r="H143" s="0" t="inlineStr">
+        <is>
+          <t>Qualidade</t>
+        </is>
+      </c>
+      <c r="I143" s="0" t="inlineStr">
+        <is>
+          <t>Em andamento</t>
+        </is>
+      </c>
+      <c r="J143" s="0">
+        <v>4</v>
+      </c>
+      <c r="K143" s="0" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="L143" s="0" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="M143" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="N143" s="0" t="inlineStr">
+        <is>
+          <t>Matriz emulada aprovada com cinco viewports 185 estados 15 feedbacks sintéticos três experiências baralho resultado e ausência do nome do aplicativo — pendente publicar validar PostgreSQL e repetir passagem física no Chrome — Safari segue adiado</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N140"/>
+  <autoFilter ref="A1:N143"/>
   <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>
@@ -9843,11 +10041,11 @@
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>Dois jogos jogáveis</t>
+          <t>Três experiências jogáveis</t>
         </is>
       </c>
       <c r="C3" s="0">
-        <v>131</v>
+        <v>141</v>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
@@ -9856,12 +10054,12 @@
       </c>
       <c r="E3" s="0" t="inlineStr">
         <is>
-          <t>Jornadas completas com lote mínimo e feedback no produto</t>
+          <t>Dois jogos amostra autoral baralho visual e feedback funcionando</t>
         </is>
       </c>
       <c r="F3" s="0" t="inlineStr">
         <is>
-          <t>19/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="G3" s="0" t="inlineStr">
@@ -9882,7 +10080,7 @@
         </is>
       </c>
       <c r="C4" s="0">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="D4" s="0" t="inlineStr">
         <is>
@@ -9891,7 +10089,7 @@
       </c>
       <c r="E4" s="0" t="inlineStr">
         <is>
-          <t>Link controlado disponível e QA em curso com aceite físico restrito ao Chrome</t>
+          <t>Link controlado disponível e nova passagem física da versão ampliada pendente no Chrome</t>
         </is>
       </c>
       <c r="F4" s="0" t="inlineStr">
@@ -10463,7 +10661,7 @@
       </c>
       <c r="F4" s="0" t="inlineStr">
         <is>
-          <t>Revisão por especialista e avisos claros de caráter educativo</t>
+          <t>Amostra autoral com aviso não oficial e não diagnóstico — manter revisão especializada antes de ampliar</t>
         </is>
       </c>
       <c r="G4" s="0" t="inlineStr">
@@ -10967,7 +11165,7 @@
       </c>
       <c r="F16" s="0" t="inlineStr">
         <is>
-          <t>Bloquear novas áreas no teste e exigir a retirada de um item para qualquer inclusão</t>
+          <t>Ampliação autorizada pela Product Owner em 17/09/2026 — separar sinais por experiência e exigir revalidação física antes dos cinco casais</t>
         </is>
       </c>
       <c r="G16" s="0" t="inlineStr">
@@ -10977,7 +11175,7 @@
       </c>
       <c r="H16" s="0" t="inlineStr">
         <is>
-          <t>Aberto</t>
+          <t>Em acompanhamento</t>
         </is>
       </c>
     </row>
@@ -11093,7 +11291,7 @@
       </c>
       <c r="F19" s="0" t="inlineStr">
         <is>
-          <t>Equilibrar duração tema e quantidade de cartas entre os dois jogos</t>
+          <t>Analisar feedback separadamente entre os dois jogos e a amostra autoral para não misturar efeito de conteúdo e interação</t>
         </is>
       </c>
       <c r="G19" s="0" t="inlineStr">

</xml_diff>

<commit_message>
registra publicacao da iteracao ampliada
</commit_message>
<xml_diff>
--- a/Plano de trabalho/acompanhamento-app-do-amor.xlsx
+++ b/Plano de trabalho/acompanhamento-app-do-amor.xlsx
@@ -109,7 +109,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>17/09/2026 12:29</t>
+          <t>17/09/2026 12:33</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -9469,7 +9469,7 @@
       </c>
       <c r="L136" s="0" t="inlineStr">
         <is>
-          <t>16/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="M136" s="3">
@@ -9477,7 +9477,7 @@
       </c>
       <c r="N136" s="0" t="inlineStr">
         <is>
-          <t>Demonstração HTTPS publicada no Render gratuito com Web Service PostgreSQL de 1 GB sonda de saúde CORS restrito bloqueio de indexação e segredo operacional — envio persistência exportação e passagem física no Chrome validados base técnica limpa e banco expira em 16/10/2026 sem backup — Safari permanece fora da cobertura atual</t>
+          <t>Versão ampliada publicada por HTTPS no Render gratuito com três experiências baralho visual Web Service PostgreSQL de 1 GB sonda de saúde CORS restrito bloqueio de indexação e segredo operacional — novo gameId persistido e exportado base técnica limpa e banco expira em 16/10/2026 sem backup</t>
         </is>
       </c>
     </row>
@@ -9733,7 +9733,7 @@
       </c>
       <c r="L140" s="0" t="inlineStr">
         <is>
-          <t>16/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="M140" s="3">
@@ -9741,7 +9741,7 @@
       </c>
       <c r="N140" s="0" t="inlineStr">
         <is>
-          <t>POST anônimo com validação idempotência controle de origem rate limit armazenamento PostgreSQL remoto com fallback JSON local e exportação CSV protegida por token — concluído em 16/09/2026</t>
+          <t>POST anônimo com validação idempotência controle de origem rate limit armazenamento PostgreSQL remoto fallback JSON local e exportação CSV protegida — schema ampliado e validado ao vivo para love-style-sample em 17/09/2026 sem armazenar respostas ou resultado</t>
         </is>
       </c>
     </row>
@@ -9939,7 +9939,7 @@
       </c>
       <c r="N143" s="0" t="inlineStr">
         <is>
-          <t>Matriz emulada aprovada com cinco viewports 185 estados 15 feedbacks sintéticos três experiências baralho resultado e ausência do nome do aplicativo — pendente publicar validar PostgreSQL e repetir passagem física no Chrome — Safari segue adiado</t>
+          <t>Versão ampliada publicada e aprovada em cinco viewports 185 estados 15 feedbacks sintéticos três experiências baralho resultado nome oculto PostgreSQL e exportação ao vivo — registro técnico removido e acesso externo ao banco fechado — pendente somente repetir a passagem física no Chrome — Safari segue adiado</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
configura pipeline de integracao continua
</commit_message>
<xml_diff>
--- a/Plano de trabalho/acompanhamento-app-do-amor.xlsx
+++ b/Plano de trabalho/acompanhamento-app-do-amor.xlsx
@@ -109,7 +109,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>17/09/2026 12:33</t>
+          <t>17/09/2026 16:44</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -3186,7 +3186,7 @@
       </c>
       <c r="I41" s="0" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="J41" s="0">
@@ -3194,7 +3194,7 @@
       </c>
       <c r="K41" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="L41" s="0" t="inlineStr">
@@ -3203,11 +3203,11 @@
         </is>
       </c>
       <c r="M41" s="3">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="N41" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>Workflow GitHub Actions criado em .github/workflows/ci.yml com Ubuntu 24.04 Node 24.20.0 cache npm instalação por lockfile permissões somente leitura concorrência timeout e gates de lint formato build OpenAPI ameaças LGPD feedback produção matriz móvel e planilha — documentação em docs/INTEGRACAO-CONTINUA.md — aguarda primeira execução remota aprovada</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
conclui tarefa de integracao continua
</commit_message>
<xml_diff>
--- a/Plano de trabalho/acompanhamento-app-do-amor.xlsx
+++ b/Plano de trabalho/acompanhamento-app-do-amor.xlsx
@@ -109,7 +109,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>17/09/2026 16:44</t>
+          <t>17/09/2026 16:55</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -3186,7 +3186,7 @@
       </c>
       <c r="I41" s="0" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="J41" s="0">
@@ -3199,15 +3199,15 @@
       </c>
       <c r="L41" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="M41" s="3">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="N41" s="0" t="inlineStr">
         <is>
-          <t>Workflow GitHub Actions criado em .github/workflows/ci.yml com Ubuntu 24.04 Node 24.20.0 cache npm instalação por lockfile permissões somente leitura concorrência timeout e gates de lint formato build OpenAPI ameaças LGPD feedback produção matriz móvel e planilha — documentação em docs/INTEGRACAO-CONTINUA.md — aguarda primeira execução remota aprovada</t>
+          <t>Workflow GitHub Actions em .github/workflows/ci.yml com Ubuntu 24.04 Node 24.20.0 cache npm instalação por lockfile permissões somente leitura concorrência timeout e gates de lint formato build OpenAPI ameaças LGPD feedback produção matriz móvel e planilha — documentação em docs/INTEGRACAO-CONTINUA.md — execução remota 1 aprovada em https://github.com/tatyelopes/APPDOAMOR/actions/runs/35267092012</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
estrutura postgres local e migracoes
</commit_message>
<xml_diff>
--- a/Plano de trabalho/acompanhamento-app-do-amor.xlsx
+++ b/Plano de trabalho/acompanhamento-app-do-amor.xlsx
@@ -109,7 +109,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>17/09/2026 16:55</t>
+          <t>17/09/2026 17:12</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -3260,7 +3260,7 @@
       </c>
       <c r="K42" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>16/09/2026</t>
         </is>
       </c>
       <c r="L42" s="0" t="inlineStr">
@@ -3273,7 +3273,7 @@
       </c>
       <c r="N42" s="0" t="inlineStr">
         <is>
-          <t>Adaptador DATABASE_URL e schema idempotente implementados para o feedback do MPV em 16/09/2026 com PostgreSQL gratuito temporário no Render - ainda provisionar local staging e production definitivos com identidades distintas migrações integridade concorrência e migração dos demais dados</t>
+          <t>PostgreSQL gratuito temporário do feedback ativo no Render — em 17/09/2026 foram adicionados PostgreSQL 18 local via Compose executor transacional com lock e checksum duas migrações versionadas para 12 tabelas de domínio mais schema_migrations e validação real no CI — ainda integrar cadastro casal sessões respostas e analytics migrar dados legados com reconciliação e provisionar homologação e produção definitivas isoladas</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
registra validacao das migracoes postgres
</commit_message>
<xml_diff>
--- a/Plano de trabalho/acompanhamento-app-do-amor.xlsx
+++ b/Plano de trabalho/acompanhamento-app-do-amor.xlsx
@@ -109,7 +109,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>17/09/2026 17:12</t>
+          <t>17/09/2026 17:19</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -3273,7 +3273,7 @@
       </c>
       <c r="N42" s="0" t="inlineStr">
         <is>
-          <t>PostgreSQL gratuito temporário do feedback ativo no Render — em 17/09/2026 foram adicionados PostgreSQL 18 local via Compose executor transacional com lock e checksum duas migrações versionadas para 12 tabelas de domínio mais schema_migrations e validação real no CI — ainda integrar cadastro casal sessões respostas e analytics migrar dados legados com reconciliação e provisionar homologação e produção definitivas isoladas</t>
+          <t>PostgreSQL gratuito temporário do feedback ativo no Render — em 17/09/2026 foram adicionados PostgreSQL 18 local via Compose executor transacional com lock e checksum duas migrações versionadas para 12 tabelas de domínio mais schema_migrations e validação real aprovada em https://github.com/tatyelopes/APPDOAMOR/actions/runs/35269876662 — ainda integrar cadastro casal sessões respostas e analytics migrar dados legados com reconciliação e provisionar homologação e produção definitivas isoladas</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
adiciona gestao segura de segredos
</commit_message>
<xml_diff>
--- a/Plano de trabalho/acompanhamento-app-do-amor.xlsx
+++ b/Plano de trabalho/acompanhamento-app-do-amor.xlsx
@@ -109,7 +109,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>17/09/2026 17:19</t>
+          <t>17/09/2026 17:39</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -3318,7 +3318,7 @@
       </c>
       <c r="I43" s="0" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="J43" s="0">
@@ -3326,7 +3326,7 @@
       </c>
       <c r="K43" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="L43" s="0" t="inlineStr">
@@ -3335,11 +3335,11 @@
         </is>
       </c>
       <c r="M43" s="3">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="N43" s="0" t="inlineStr">
         <is>
-          <t>Cofre identidades e chaves exclusivos por ambiente conforme docs/AMBIENTES.md - injeção em runtime privilégio mínimo inventário rotação e auditoria - modelos e gitignore não substituem esses controles</t>
+          <t>Baseline gratuita implementada em docs/GESTAO-DE-SEGREDOS.md com inventário matriz por ambiente geração local criptograficamente aleatória sem exibição validação fail-closed em runtime scanner de arquivos rastreados e staged hook pre-commit gate no CI modelo de rotação e injeção atual do Render — pendentes cofres e identidades definitivos de homologação e produção responsáveis nominais e primeira rotação comprovada</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
registra validacao da gestao de segredos
</commit_message>
<xml_diff>
--- a/Plano de trabalho/acompanhamento-app-do-amor.xlsx
+++ b/Plano de trabalho/acompanhamento-app-do-amor.xlsx
@@ -109,7 +109,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>17/09/2026 17:39</t>
+          <t>17/09/2026 17:44</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -3339,7 +3339,7 @@
       </c>
       <c r="N43" s="0" t="inlineStr">
         <is>
-          <t>Baseline gratuita implementada em docs/GESTAO-DE-SEGREDOS.md com inventário matriz por ambiente geração local criptograficamente aleatória sem exibição validação fail-closed em runtime scanner de arquivos rastreados e staged hook pre-commit gate no CI modelo de rotação e injeção atual do Render — pendentes cofres e identidades definitivos de homologação e produção responsáveis nominais e primeira rotação comprovada</t>
+          <t>Baseline gratuita implementada em docs/GESTAO-DE-SEGREDOS.md com inventário matriz por ambiente geração local criptograficamente aleatória sem exibição validação fail-closed em runtime scanner de arquivos rastreados staged e histórico hook pre-commit gate aprovado em https://github.com/tatyelopes/APPDOAMOR/actions/runs/35272382976 modelo de rotação e injeção atual do Render — pendentes cofres e identidades definitivos de homologação e produção responsáveis nominais e primeira rotação comprovada</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
aplica migracoes ao iniciar a api
</commit_message>
<xml_diff>
--- a/Plano de trabalho/acompanhamento-app-do-amor.xlsx
+++ b/Plano de trabalho/acompanhamento-app-do-amor.xlsx
@@ -109,7 +109,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>17/09/2026 17:44</t>
+          <t>17/09/2026 20:43</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -3273,7 +3273,7 @@
       </c>
       <c r="N42" s="0" t="inlineStr">
         <is>
-          <t>PostgreSQL gratuito temporário do feedback ativo no Render — em 17/09/2026 foram adicionados PostgreSQL 18 local via Compose executor transacional com lock e checksum duas migrações versionadas para 12 tabelas de domínio mais schema_migrations e validação real aprovada em https://github.com/tatyelopes/APPDOAMOR/actions/runs/35269876662 — ainda integrar cadastro casal sessões respostas e analytics migrar dados legados com reconciliação e provisionar homologação e produção definitivas isoladas</t>
+          <t>PostgreSQL gratuito temporário do feedback ativo no Render — em 17/09/2026 foram adicionados PostgreSQL 18 local via Compose executor transacional com lock e checksum duas migrações versionadas para 12 tabelas de domínio mais schema_migrations validação real aprovada em https://github.com/tatyelopes/APPDOAMOR/actions/runs/35269876662 e bootstrap automático da API para aplicar migrações antes de aceitar tráfego — ainda integrar cadastro casal sessões respostas e analytics migrar dados legados com reconciliação e provisionar homologação e produção definitivas isoladas</t>
         </is>
       </c>
     </row>
@@ -3339,7 +3339,7 @@
       </c>
       <c r="N43" s="0" t="inlineStr">
         <is>
-          <t>Baseline gratuita implementada em docs/GESTAO-DE-SEGREDOS.md com inventário matriz por ambiente geração local criptograficamente aleatória sem exibição validação fail-closed em runtime scanner de arquivos rastreados staged e histórico hook pre-commit gate aprovado em https://github.com/tatyelopes/APPDOAMOR/actions/runs/35272382976 modelo de rotação e injeção atual do Render — pendentes cofres e identidades definitivos de homologação e produção responsáveis nominais e primeira rotação comprovada</t>
+          <t>Baseline gratuita implementada em docs/GESTAO-DE-SEGREDOS.md com inventário matriz por ambiente geração local criptograficamente aleatória sem exibição validação fail-closed em runtime scanner de arquivos rastreados staged e histórico hook pre-commit gate aprovado em https://github.com/tatyelopes/APPDOAMOR/actions/runs/35272382976 modelo de rotação e injeção atual do Render — token de exportação do MPV rotacionado em 17/09/2026 após exposição acidental e salvo localmente sem exibição — pendentes cofres e identidades definitivos de homologação e produção e responsáveis nominais</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
registra exportacao ao vivo do feedback
</commit_message>
<xml_diff>
--- a/Plano de trabalho/acompanhamento-app-do-amor.xlsx
+++ b/Plano de trabalho/acompanhamento-app-do-amor.xlsx
@@ -109,7 +109,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>17/09/2026 20:43</t>
+          <t>17/09/2026 20:50</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -3273,7 +3273,7 @@
       </c>
       <c r="N42" s="0" t="inlineStr">
         <is>
-          <t>PostgreSQL gratuito temporário do feedback ativo no Render — em 17/09/2026 foram adicionados PostgreSQL 18 local via Compose executor transacional com lock e checksum duas migrações versionadas para 12 tabelas de domínio mais schema_migrations validação real aprovada em https://github.com/tatyelopes/APPDOAMOR/actions/runs/35269876662 e bootstrap automático da API para aplicar migrações antes de aceitar tráfego — ainda integrar cadastro casal sessões respostas e analytics migrar dados legados com reconciliação e provisionar homologação e produção definitivas isoladas</t>
+          <t>PostgreSQL gratuito temporário do feedback ativo no Render — em 17/09/2026 foram adicionados PostgreSQL 18 local via Compose executor transacional com lock e checksum duas migrações versionadas para 12 tabelas de domínio mais schema_migrations validação real aprovada em https://github.com/tatyelopes/APPDOAMOR/actions/runs/35269876662 e bootstrap automático da API aprovado no CI em https://github.com/tatyelopes/APPDOAMOR/actions/runs/35288177777 — após novo deploy a migração automática e a exportação protegida foram confirmadas ao vivo com base vazia — ainda integrar cadastro casal sessões respostas e analytics migrar dados legados com reconciliação e provisionar homologação e produção definitivas isoladas</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
adiciona arquivos do projeto
</commit_message>
<xml_diff>
--- a/Plano de trabalho/acompanhamento-app-do-amor.xlsx
+++ b/Plano de trabalho/acompanhamento-app-do-amor.xlsx
@@ -109,7 +109,7 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>17/09/2026 21:09</t>
+          <t>23/09/2026 22:38</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -142,7 +142,7 @@
         </is>
       </c>
       <c r="B4" s="2">
-        <f>COUNTA('Plano Mestre'!A2:A143)</f>
+        <f>COUNTA('Plano Mestre'!A2:A145)</f>
         <v>0</v>
       </c>
       <c r="C4" s="0" t="inlineStr">
@@ -158,7 +158,7 @@
         </is>
       </c>
       <c r="B5" s="2">
-        <f>COUNTIF('Plano Mestre'!I2:I143,"Concluído")</f>
+        <f>COUNTIF('Plano Mestre'!I2:I145,"Concluído")</f>
         <v>0</v>
       </c>
       <c r="C5" s="0" t="inlineStr">
@@ -174,7 +174,7 @@
         </is>
       </c>
       <c r="B6" s="2">
-        <f>COUNTIF('Plano Mestre'!I2:I143,"Em andamento")</f>
+        <f>COUNTIF('Plano Mestre'!I2:I145,"Em andamento")</f>
         <v>0</v>
       </c>
       <c r="C6" s="0" t="inlineStr">
@@ -190,7 +190,7 @@
         </is>
       </c>
       <c r="B7" s="2">
-        <f>COUNTIF('Plano Mestre'!I2:I143,"Não iniciado")</f>
+        <f>COUNTIF('Plano Mestre'!I2:I145,"Não iniciado")</f>
         <v>0</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
@@ -206,7 +206,7 @@
         </is>
       </c>
       <c r="B8" s="3">
-        <f>AVERAGE('Plano Mestre'!M2:M143)</f>
+        <f>AVERAGE('Plano Mestre'!M2:M145)</f>
         <v>0</v>
       </c>
       <c r="C8" s="0" t="inlineStr">
@@ -222,7 +222,7 @@
         </is>
       </c>
       <c r="B9" s="2">
-        <f>SUM('Plano Mestre'!J2:J143)</f>
+        <f>SUM('Plano Mestre'!J2:J145)</f>
         <v>0</v>
       </c>
       <c r="C9" s="0" t="inlineStr">
@@ -272,11 +272,11 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B143,"Descoberta")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B145,"Descoberta")</f>
         <v>0</v>
       </c>
       <c r="C12" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B143,"Descoberta",'Plano Mestre'!I2:I143,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B145,"Descoberta",'Plano Mestre'!I2:I145,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -287,11 +287,11 @@
         </is>
       </c>
       <c r="B13" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B143,"Planejamento")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B145,"Planejamento")</f>
         <v>0</v>
       </c>
       <c r="C13" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B143,"Planejamento",'Plano Mestre'!I2:I143,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B145,"Planejamento",'Plano Mestre'!I2:I145,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -302,11 +302,11 @@
         </is>
       </c>
       <c r="B14" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B143,"Marca")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B145,"Marca")</f>
         <v>0</v>
       </c>
       <c r="C14" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B143,"Marca",'Plano Mestre'!I2:I143,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B145,"Marca",'Plano Mestre'!I2:I145,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -317,11 +317,11 @@
         </is>
       </c>
       <c r="B15" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B143,"UX/UI")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B145,"UX/UI")</f>
         <v>0</v>
       </c>
       <c r="C15" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B143,"UX/UI",'Plano Mestre'!I2:I143,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B145,"UX/UI",'Plano Mestre'!I2:I145,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -332,11 +332,11 @@
         </is>
       </c>
       <c r="B16" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B143,"Arquitetura")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B145,"Arquitetura")</f>
         <v>0</v>
       </c>
       <c r="C16" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B143,"Arquitetura",'Plano Mestre'!I2:I143,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B145,"Arquitetura",'Plano Mestre'!I2:I145,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -347,11 +347,11 @@
         </is>
       </c>
       <c r="B17" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B143,"Infraestrutura")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B145,"Infraestrutura")</f>
         <v>0</v>
       </c>
       <c r="C17" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B143,"Infraestrutura",'Plano Mestre'!I2:I143,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B145,"Infraestrutura",'Plano Mestre'!I2:I145,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -362,11 +362,11 @@
         </is>
       </c>
       <c r="B18" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B143,"Backend")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B145,"Backend")</f>
         <v>0</v>
       </c>
       <c r="C18" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B143,"Backend",'Plano Mestre'!I2:I143,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B145,"Backend",'Plano Mestre'!I2:I145,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -377,11 +377,11 @@
         </is>
       </c>
       <c r="B19" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B143,"Frontend")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B145,"Frontend")</f>
         <v>0</v>
       </c>
       <c r="C19" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B143,"Frontend",'Plano Mestre'!I2:I143,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B145,"Frontend",'Plano Mestre'!I2:I145,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -392,11 +392,11 @@
         </is>
       </c>
       <c r="B20" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B143,"Conteúdo")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B145,"Conteúdo")</f>
         <v>0</v>
       </c>
       <c r="C20" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B143,"Conteúdo",'Plano Mestre'!I2:I143,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B145,"Conteúdo",'Plano Mestre'!I2:I145,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -407,11 +407,11 @@
         </is>
       </c>
       <c r="B21" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B143,"Qualidade")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B145,"Qualidade")</f>
         <v>0</v>
       </c>
       <c r="C21" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B143,"Qualidade",'Plano Mestre'!I2:I143,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B145,"Qualidade",'Plano Mestre'!I2:I145,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -422,11 +422,11 @@
         </is>
       </c>
       <c r="B22" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B143,"Jurídico")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B145,"Jurídico")</f>
         <v>0</v>
       </c>
       <c r="C22" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B143,"Jurídico",'Plano Mestre'!I2:I143,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B145,"Jurídico",'Plano Mestre'!I2:I145,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -437,11 +437,11 @@
         </is>
       </c>
       <c r="B23" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B143,"Lançamento")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B145,"Lançamento")</f>
         <v>0</v>
       </c>
       <c r="C23" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B143,"Lançamento",'Plano Mestre'!I2:I143,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B145,"Lançamento",'Plano Mestre'!I2:I145,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -452,11 +452,11 @@
         </is>
       </c>
       <c r="B24" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B143,"Pós-lançamento")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B145,"Pós-lançamento")</f>
         <v>0</v>
       </c>
       <c r="C24" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B143,"Pós-lançamento",'Plano Mestre'!I2:I143,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B145,"Pós-lançamento",'Plano Mestre'!I2:I145,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -467,11 +467,11 @@
         </is>
       </c>
       <c r="B25" s="2">
-        <f>COUNTIF('Plano Mestre'!B2:B143,"MPV de teste")</f>
+        <f>COUNTIF('Plano Mestre'!B2:B145,"MPV de teste")</f>
         <v>0</v>
       </c>
       <c r="C25" s="2">
-        <f>COUNTIFS('Plano Mestre'!B2:B143,"MPV de teste",'Plano Mestre'!I2:I143,"Concluído")</f>
+        <f>COUNTIFS('Plano Mestre'!B2:B145,"MPV de teste",'Plano Mestre'!I2:I145,"Concluído")</f>
         <v>0</v>
       </c>
     </row>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="N25" s="0" t="inlineStr">
         <is>
-          <t>Desenho em docs/HOME-E-ROTINA-DIARIA.md e protótipo navegável em docs/prototipo-home-rotina.html - 13 estados da home e rotina com perguntas desafios e modo misto - pendentes revisão visual e validação com casais na tarefa 30</t>
+          <t>Desenho em docs/HOME-E-ROTINA-DIARIA.md e protótipo navegável em docs/prototipo-home-rotina.html - 13 estados da home e rotina com perguntas desafios e modo misto - home do casal conectado aprovada visualmente pela Product Owner em 23/09/2026 com as quatro dinâmicas de Explorem juntos acima do cartão Gesto de hoje - pendente validação com casais na tarefa 30</t>
         </is>
       </c>
     </row>
@@ -2217,7 +2217,7 @@
       </c>
       <c r="N26" s="0" t="inlineStr">
         <is>
-          <t>Desenho em docs/PERGUNTAS-E-REVELACAO-MUTUA.md e protótipo docs/prototipo-perguntas-revelacao.html - discursiva múltipla escolha desafios espera correção pulo retomada e revelação bilateral - verificação de estados automatizada - validação visual e com casais pendentes na tarefa 30</t>
+          <t>Desenho em docs/PERGUNTAS-E-REVELACAO-MUTUA.md e protótipo docs/prototipo-perguntas-revelacao.html - discursiva múltipla escolha desafios espera correção pulo retomada e revelação bilateral - durante a revisão de 23/09/2026 a configuração recebeu seleção de temas por cápsulas quarto formato Múltipla escolha funcional e níveis Leve e Profunda com conteúdo ilustrativo do protótipo - verificação de estados automatizada - validação visual da configuração rodada e com casais pendentes na tarefa 30</t>
         </is>
       </c>
     </row>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="N27" s="0" t="inlineStr">
         <is>
-          <t>Desenho em docs/TESTES-E-RESULTADOS.md e protótipo docs/prototipo-testes-resultados.html - formas de afeto e temperamentos experimentais com pausa revisão resultado parcial empate compartilhamento opcional e revogação - verificação de estados em scripts/validate-tests-prototype.mjs - revisão visual editorial especializada e validação com casais pendentes</t>
+          <t>Desenho em docs/TESTES-E-RESULTADOS.md e protótipo docs/prototipo-testes-resultados.html - formas de afeto e temperamentos experimentais com pausa revisão resultado parcial empate compartilhamento opcional e revogação - as 32 combinações da implementação binária atual foram mapeadas em Conteúdo/mapeamento-linguagens-do-amor.xlsx com gerador e validador próprios - o mapeamento evidenciou desempate atual por primeira ocorrência divergente da regra TR-11 e pendente de decisão editorial - revisão visual especializada e validação com casais pendentes</t>
         </is>
       </c>
     </row>
@@ -2332,11 +2332,11 @@
         </is>
       </c>
       <c r="J28" s="0">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="K28" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>21/09/2026</t>
         </is>
       </c>
       <c r="L28" s="0" t="inlineStr">
@@ -2349,7 +2349,7 @@
       </c>
       <c r="N28" s="0" t="inlineStr">
         <is>
-          <t>Home rotina diária perguntas com revelação e testes com resultados desenhados em protótipos HTML responsivos na pasta docs - demais telas e validação visual completa pendentes</t>
+          <t>Revisão página por página iniciada em 21/09/2026 - onboarding cadastro pareamento convite Home Correio do Amor e Perfil aprovados visualmente pela Product Owner até 23/09/2026 - configuração de Perguntas que aproximam recebeu Múltipla escolha temas com corações e níveis Leve e Profunda em /wireframes/perguntas - página inicial de As linguagens do amor disponibilizada em /wireframes/linguagens-do-amor para a próxima revisão - evidências desktop e mobile em docs - primeira rodada permanece disponível em /wireframes/pergunta</t>
         </is>
       </c>
     </row>
@@ -4217,12 +4217,12 @@
       </c>
       <c r="D57" s="0" t="inlineStr">
         <is>
-          <t>Implementar linguagens do amor e resultado</t>
+          <t>Implementar formas de afeto e resultado bilateral</t>
         </is>
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
-          <t>Serviço de avaliação</t>
+          <t>Serviço de avaliação e composição consentida</t>
         </is>
       </c>
       <c r="F57" s="0" t="inlineStr">
@@ -4232,7 +4232,7 @@
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>49,77</t>
         </is>
       </c>
       <c r="H57" s="0" t="inlineStr">
@@ -4246,7 +4246,7 @@
         </is>
       </c>
       <c r="J57" s="0">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="K57" s="0" t="inlineStr">
         <is>
@@ -4263,7 +4263,7 @@
       </c>
       <c r="N57" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>Manter resultado individual privado e versionado - compor visão bilateral somente quando as duas pessoas concluírem a mesma versão e compartilharem - apresentar forças complementaridades oportunidades e sugestões aprovadas sem nota de compatibilidade - revogação ou desvinculação encerra acesso</t>
         </is>
       </c>
     </row>
@@ -4364,7 +4364,7 @@
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>49,56</t>
         </is>
       </c>
       <c r="H59" s="0" t="inlineStr">
@@ -4395,7 +4395,7 @@
       </c>
       <c r="N59" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>Incluir sugestão semanal derivada do resultado bilateral somente por opt-in individual - frequência dia horário pausa e desligamento configuráveis - cancelar ao revogar compartilhamento ou vínculo - payload de push neutro sem resultado ou tema íntimo</t>
         </is>
       </c>
     </row>
@@ -4646,7 +4646,7 @@
       </c>
       <c r="K63" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>22/09/2026</t>
         </is>
       </c>
       <c r="L63" s="0" t="inlineStr">
@@ -4659,7 +4659,7 @@
       </c>
       <c r="N63" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>Layout de cadastro aprovado pela Product Owner em 22/09/2026 na rota /wireframes/cadastro com chamada removida título em duas linhas e estrela dourada - integração funcional existente preservada - modo de login permanece pendente de revisão</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
       </c>
       <c r="K64" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>22/09/2026</t>
         </is>
       </c>
       <c r="L64" s="0" t="inlineStr">
@@ -4725,7 +4725,7 @@
       </c>
       <c r="N64" s="0" t="inlineStr">
         <is>
-          <t>Criação entrada e espera implementadas - reaberto na revisão: erro de atualização sem mensagem e cópia pode informar sucesso sem clipboard - integração e validação completas pendentes</t>
+          <t>Criação entrada e espera implementadas - telas de escolha e de convite e espera aprovadas visualmente pela Product Owner em 23/09/2026 nas rotas /wireframes/conectar e /wireframes/convite - indicadores das três etapas ampliados e iluminados em dourado - erro de atualização sem mensagem e confirmação de cópia sem clipboard permanecem pendentes antes da validação funcional completa</t>
         </is>
       </c>
     </row>
@@ -4791,7 +4791,7 @@
       </c>
       <c r="N65" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>Tela atual de conta vínculo código do casal atualização e saída aprovada visualmente pela Product Owner em 23/09/2026 na rota /wireframes/perfil - preferências privacidade e gestão de vínculo previstas no escopo completo permanecem pendentes</t>
         </is>
       </c>
     </row>
@@ -4857,7 +4857,7 @@
       </c>
       <c r="N66" s="0" t="inlineStr">
         <is>
-          <t>Home atual parcial - integrar estados em docs/HOME-E-ROTINA-DIARIA.md com pendências reais e progresso confirmado sem valores demonstrativos</t>
+          <t>Home atual parcial aprovada visualmente pela Product Owner em 23/09/2026 na rota /wireframes/home com Explorem juntos e as quatro dinâmicas primeiro e Gesto de hoje abaixo sem duplicação - ainda integrar estados em docs/HOME-E-ROTINA-DIARIA.md com pendências reais e progresso confirmado sem valores demonstrativos</t>
         </is>
       </c>
     </row>
@@ -4906,7 +4906,7 @@
         </is>
       </c>
       <c r="J67" s="0">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K67" s="0" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="N67" s="0" t="inlineStr">
         <is>
-          <t>Jogo local por temas implementado em 109 - níveis leve médio profundo e catálogo remoto ainda pendentes - harmonizar formato e mecânica na tarefa 112</t>
+          <t>Configuração do jogo local em /wireframes/perguntas ajustada em 23/09/2026 com temas em cápsulas selecionáveis escolha funcional entre Leve e Profunda quatro formatos em grade e Múltipla escolha com seleção e confirmação separadas - o nível altera perguntas desafios e alternativas da sessão - conteúdo atual é ilustrativo e aguarda aprovação editorial da tarefa 108 - catálogo remoto e harmonização na tarefa 112 permanecem pendentes</t>
         </is>
       </c>
     </row>
@@ -5075,7 +5075,7 @@
       </c>
       <c r="D70" s="0" t="inlineStr">
         <is>
-          <t>Implementar teste de linguagens do amor</t>
+          <t>Implementar formas de afeto e visão bilateral</t>
         </is>
       </c>
       <c r="E70" s="0" t="inlineStr">
@@ -5104,7 +5104,7 @@
         </is>
       </c>
       <c r="J70" s="0">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="K70" s="0" t="inlineStr">
         <is>
@@ -5121,7 +5121,7 @@
       </c>
       <c r="N70" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>Primeira pergunta da experiência individual disponibilizada para revisão visual em /wireframes/linguagens-do-amor em 23/09/2026 - lógica binária atual documentada em planilha com 32 combinações pontuações empates e resultados - desempate por primeira ocorrência deve ser substituído ou aprovado editorialmente antes da validação - preservar resultado individual e compartilhamento explícito - após duas conclusões compatíveis apresentar forças compartilhadas formas complementares oportunidades de cuidado e sugestões do que cada pessoa pode experimentar pela outra - sem diagnóstico déficit ou nota de compatibilidade</t>
         </is>
       </c>
     </row>
@@ -5288,7 +5288,7 @@
       </c>
       <c r="G73" s="0" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>58,69</t>
         </is>
       </c>
       <c r="H73" s="0" t="inlineStr">
@@ -5302,7 +5302,7 @@
         </is>
       </c>
       <c r="J73" s="0">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="K73" s="0" t="inlineStr">
         <is>
@@ -5319,7 +5319,7 @@
       </c>
       <c r="N73" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>Oferecer ativação individual de sugestão semanal após visão bilateral - permitir configurar pausar e desligar - push neutro abre conteúdo apenas após autenticação e não registra gesto como prova ou progresso</t>
         </is>
       </c>
     </row>
@@ -5632,7 +5632,7 @@
         </is>
       </c>
       <c r="J78" s="0">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="K78" s="0" t="inlineStr">
         <is>
@@ -5649,7 +5649,7 @@
       </c>
       <c r="N78" s="0" t="inlineStr">
         <is>
-          <t>Validar lotes e recomendações antes de publicação - distinguir conteúdo candidato de aprovado e seleção mínima de 60 atividades - conteúdo íntimo restrito conforme baseline do piloto</t>
+          <t>Produzir matriz candidata e validar sugestões de cuidado por combinação de formas de afeto além dos lotes de atividades - recomendações devem ser pequenas adaptáveis e orientadas pela preferência de quem recebe - distinguir conteúdo candidato de aprovado - seleção mínima de 60 atividades e conteúdo íntimo restrito conforme baseline</t>
         </is>
       </c>
     </row>
@@ -6872,7 +6872,7 @@
       </c>
       <c r="G97" s="0" t="inlineStr">
         <is>
-          <t>87,90,92-95,77,116,117,119,121,122</t>
+          <t>87,90,92-95,77,116,117,119,121,122,143</t>
         </is>
       </c>
       <c r="H97" s="0" t="inlineStr">
@@ -6903,7 +6903,7 @@
       </c>
       <c r="N97" s="0" t="inlineStr">
         <is>
-          <t>UAT do ciclo bilateral conforme baseline 112 - mecânicas 113 e 114 entram no aceite se mantidas para o piloto - reunir evidências de conteúdo privacidade fornecedores e operação</t>
+          <t>UAT do ciclo bilateral conforme baseline 112 - mecânicas 113 e 114 entram no aceite do primeiro piloto - resultado bilateral e lembrete semanal da tarefa 143 são obrigatórios para o aceite pré-lançamento - reunir evidências de conteúdo privacidade fornecedores e operação</t>
         </is>
       </c>
     </row>
@@ -7695,7 +7695,7 @@
       </c>
       <c r="N109" s="0" t="inlineStr">
         <is>
-          <t>75 perguntas de múltipla escolha candidatas em Conteúdo/banco-de-perguntas-conectadois.xlsx - produção precede revisão 76 e parecer 77 - pendentes revisão editorial aprovação e seleção do lote do piloto</t>
+          <t>75 perguntas de múltipla escolha candidatas em Conteúdo/banco-de-perguntas-conectadois.xlsx - interface funcional usa temporariamente pergunta e quatro alternativas ilustrativas já definidas no protótipo sem promover conteúdo candidato - produção precede revisão 76 e parecer 77 - pendentes revisão editorial aprovação e seleção do lote do piloto</t>
         </is>
       </c>
     </row>
@@ -7761,7 +7761,7 @@
       </c>
       <c r="N110" s="0" t="inlineStr">
         <is>
-          <t>Onze temas com dois formatos e modo misto - respostas por jogador e confirmação individual de desafios - pular e reiniciar disponíveis</t>
+          <t>Onze temas apresentados em cápsulas responsivas com ícones de coração seleção de nível Leve ou Profunda e quatro formatos Perguntas discursivas Múltipla escolha Desafios e modo misto - múltipla escolha exige seleção seguida de confirmação - respostas por jogador confirmação individual de desafios pular e reiniciar disponíveis - configuração ajustada em /wireframes/perguntas em 23/09/2026</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="I112" s="0" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="J112" s="0">
@@ -7880,7 +7880,7 @@
       </c>
       <c r="K112" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>21/09/2026</t>
         </is>
       </c>
       <c r="L112" s="0" t="inlineStr">
@@ -7889,11 +7889,11 @@
         </is>
       </c>
       <c r="M112" s="3">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="N112" s="0" t="inlineStr">
         <is>
-          <t>Implementar modelo de partidas e snapshots de conteúdo - integrar respostas e progresso com transações e testes de concorrência</t>
+          <t>Primeira fatia em /api/v1/game-sessions cria e retoma partidas autenticadas com idempotência isolamento por casal participantes e snapshots do catálogo atual - validação ponta a ponta em scripts/validate-game-sessions.mjs e contrato marcado como parcial - pendentes persistência PostgreSQL respostas progresso transacional retomada no frontend e testes de concorrência</t>
         </is>
       </c>
     </row>
@@ -7938,7 +7938,7 @@
       </c>
       <c r="I113" s="0" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="J113" s="0">
@@ -7946,20 +7946,20 @@
       </c>
       <c r="K113" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>21/09/2026</t>
         </is>
       </c>
       <c r="L113" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>21/09/2026</t>
         </is>
       </c>
       <c r="M113" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N113" s="0" t="inlineStr">
         <is>
-          <t>Conciliar perguntas desafios e misto com resposta guardada adivinhação e coincidências - decidir primeiro piloto e atualizar PRD escopo MoSCoW modelo e cronograma - estimativa preliminar</t>
+          <t>Baseline aprovada em docs/DECISAO-ESCOPO-PILOTO-2026-09-21.md - primeiro piloto inclui três níveis perguntas desafios modo misto e desafio na adivinhação - resultado bilateral e lembrete semanal ficam na iteração seguinte pela tarefa 143 e são obrigatórios antes da UAT e do lançamento - PRD escopo MoSCoW e rastreabilidade atualizados</t>
         </is>
       </c>
     </row>
@@ -8008,7 +8008,7 @@
         </is>
       </c>
       <c r="J114" s="0">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="K114" s="0" t="inlineStr">
         <is>
@@ -8025,7 +8025,7 @@
       </c>
       <c r="N114" s="0" t="inlineStr">
         <is>
-          <t>Já previsto no escopo MVP - execução condicionada à decisão 112 - incluir modelo de tentativas API interface e testes de autoria - estimativa preliminar</t>
+          <t>Incluir perguntas de preferência e variação de gesto ou desafio desejado - palpite e revelação separados do aceite bilateral para executar adaptar trocar ou pular sem prova - incluir modelo de tentativas API interface autoria consentimento e testes - execução condicionada à baseline 112</t>
         </is>
       </c>
     </row>
@@ -9512,7 +9512,7 @@
       </c>
       <c r="G137" s="0" t="inlineStr">
         <is>
-          <t>135,142</t>
+          <t>135</t>
         </is>
       </c>
       <c r="H137" s="0" t="inlineStr">
@@ -9522,7 +9522,7 @@
       </c>
       <c r="I137" s="0" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="J137" s="0">
@@ -9539,11 +9539,11 @@
         </is>
       </c>
       <c r="M137" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N137" s="0" t="inlineStr">
         <is>
-          <t>Cada casal usa as experiências sem mediação e envia os três sinais do produto com sugestão de melhoria opcional — não há entrevistas nem etapa de pesquisa dentro do MPV — iniciar após a nova passagem física da versão ampliada</t>
+          <t>Validação com cinco casais aceita como concluída pela Product Owner em 21/09/2026 - decisão e limites registrados em docs/VALIDACAO-MPV-CINCO-CASAIS-2026-09-21.md - continuar o formato com ajustes - os comentários qualitativos foram aceitos como achados da rodada e os 5 sinais anônimos da API permanecem apenas como evidência agregada - a passagem física 142 segue como hardening de qualidade sem bloquear este aceite</t>
         </is>
       </c>
     </row>
@@ -9588,7 +9588,7 @@
       </c>
       <c r="I138" s="0" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="J138" s="0">
@@ -9605,11 +9605,11 @@
         </is>
       </c>
       <c r="M138" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N138" s="0" t="inlineStr">
         <is>
-          <t>Registrar continuar ajustar ou encerrar o formato e quais evidências devem orientar a futura revisão do plano completo sem alterá-lo automaticamente</t>
+          <t>Concluído em 21/09/2026 com registro em docs/FEEDBACK-DE-PRODUTO-2026-09-21.md e docs/VALIDACAO-MPV-CINCO-CASAIS-2026-09-21.md - PRD escopo fluxos e tarefas 56 58 66 69 72 77 112 e 113 atualizados - decisão de continuar o formato com ajustes sem interpretar os achados como prevalência estatística</t>
         </is>
       </c>
     </row>
@@ -9943,8 +9943,140 @@
         </is>
       </c>
     </row>
+    <row r="144">
+      <c r="A144" s="0">
+        <v>143</v>
+      </c>
+      <c r="B144" s="0" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C144" s="0" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="D144" s="0" t="inlineStr">
+        <is>
+          <t>Integrar resultado bilateral e lembrete semanal na iteração pré-lançamento</t>
+        </is>
+      </c>
+      <c r="E144" s="0" t="inlineStr">
+        <is>
+          <t>Jornada bilateral e lembrete validados</t>
+        </is>
+      </c>
+      <c r="F144" s="0" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+      <c r="G144" s="0" t="inlineStr">
+        <is>
+          <t>56,58,69,72,77,90,119</t>
+        </is>
+      </c>
+      <c r="H144" s="0" t="inlineStr">
+        <is>
+          <t>Liderança Técnica</t>
+        </is>
+      </c>
+      <c r="I144" s="0" t="inlineStr">
+        <is>
+          <t>Não iniciado</t>
+        </is>
+      </c>
+      <c r="J144" s="0">
+        <v>24</v>
+      </c>
+      <c r="K144" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L144" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M144" s="3">
+        <v>0</v>
+      </c>
+      <c r="N144" s="0" t="inlineStr">
+        <is>
+          <t>Executar depois do primeiro piloto e antes da UAT - integrar duas conclusões compatíveis compartilhamento revogável forças complementaridades oportunidades sugestões aprovadas e lembrete semanal opt-in - testar autorização desvinculação privacidade push neutro acessibilidade e cancelamento - gate obrigatório das tarefas 96 a 98 e do lançamento</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="0">
+        <v>144</v>
+      </c>
+      <c r="B145" s="0" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C145" s="0" t="inlineStr">
+        <is>
+          <t>Casal</t>
+        </is>
+      </c>
+      <c r="D145" s="0" t="inlineStr">
+        <is>
+          <t>Implementar Correio do Amor entre contas pareadas</t>
+        </is>
+      </c>
+      <c r="E145" s="0" t="inlineStr">
+        <is>
+          <t>Envio e histórico de recados do casal</t>
+        </is>
+      </c>
+      <c r="F145" s="0" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G145" s="0" t="inlineStr">
+        <is>
+          <t>27,49,63</t>
+        </is>
+      </c>
+      <c r="H145" s="0" t="inlineStr">
+        <is>
+          <t>Engenharia Frontend e Backend</t>
+        </is>
+      </c>
+      <c r="I145" s="0" t="inlineStr">
+        <is>
+          <t>Em andamento</t>
+        </is>
+      </c>
+      <c r="J145" s="0">
+        <v>16</v>
+      </c>
+      <c r="K145" s="0" t="inlineStr">
+        <is>
+          <t>23/09/2026</t>
+        </is>
+      </c>
+      <c r="L145" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M145" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="N145" s="0" t="inlineStr">
+        <is>
+          <t>Primeira fatia implementada na aba Nós e em /wireframes/correio com composição de até 280 caracteres histórico responsivo persistência no armazenamento da API autorização restrita ao casal e teste automatizado de envio e leitura pela conta parceira - visual aprovado pela Product Owner em 23/09/2026 - contrato parcial em docs/openapi-v1.json - persistência PostgreSQL definitiva permanece pendente</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N143"/>
+  <autoFilter ref="A1:N145"/>
   <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>
@@ -10119,12 +10251,12 @@
       </c>
       <c r="D5" s="0" t="inlineStr">
         <is>
-          <t>Não iniciado</t>
+          <t>Concluído</t>
         </is>
       </c>
       <c r="E5" s="0" t="inlineStr">
         <is>
-          <t>Sinais de cinco casais registrados como insumo para revisão futura do plano completo</t>
+          <t>Feedback de cinco casais registrado e incorporado ao PRD escopo fluxos e backlog</t>
         </is>
       </c>
       <c r="F5" s="0" t="inlineStr">
@@ -10134,7 +10266,7 @@
       </c>
       <c r="G5" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>21/09/2026</t>
         </is>
       </c>
     </row>
@@ -10290,7 +10422,7 @@
         </is>
       </c>
       <c r="C10" s="0">
-        <v>75</v>
+        <v>143</v>
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
@@ -10299,7 +10431,7 @@
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
-          <t>Jornada bilateral validada incluindo 111 e 116 e métricas 106-107 — 113-114 conforme decisão 112</t>
+          <t>Núcleo do primeiro piloto validado e integração pré-lançamento 143 concluída com resultado bilateral e lembrete semanal</t>
         </is>
       </c>
       <c r="F10" s="0" t="inlineStr">
@@ -10369,7 +10501,7 @@
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
-          <t>QA segurança acessibilidade privacidade UAT e restauração 118 sem bloqueador — PWA 119 validada</t>
+          <t>QA segurança acessibilidade privacidade UAT integração 143 e restauração 118 sem bloqueador — PWA 119 validada</t>
         </is>
       </c>
       <c r="F12" s="0" t="inlineStr">

</xml_diff>